<commit_message>
NEA update May 2026
</commit_message>
<xml_diff>
--- a/China NEA/review_workbooks/2024-07-25_2024年上半年光伏发电建设情况---国家能源局_review.xlsx
+++ b/China NEA/review_workbooks/2024-07-25_2024年上半年光伏发电建设情况---国家能源局_review.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,37 +444,1541 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>4960</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>5288</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1585</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>288</t>
+          <t>71293</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>1585</t>
+          <t>40342</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>71293</t>
+          <t>30951</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>40342</t>
+          <t>13184</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>108.9</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>34.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>天津</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>119.1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>20.9</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>98.3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>608.7</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>319.8</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>288.9</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>42.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>河北</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>568.2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>302.3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>265.8</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>98.2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>5984.6</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>3326.2</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2658.4</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1829.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>山西</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>352.7</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>209.8</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>142.9</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>66.6</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2843.1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2033.8</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>809.2</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>551.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>山东</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>661.2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>183.4</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>477.8</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>138.2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>6353.7</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1777.2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>4576.5</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2699.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>内蒙古</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>466.5</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>394.2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>72.2</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>43.2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2822.1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2577.2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>244.9</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>97.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>辽宁</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>149.1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>13.7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>135.4</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>95.3</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>1106.8</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>535.1</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>571.7</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>313.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>吉林</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>51.9</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>19.9</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>32.0</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>23.4</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>511.7</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>360.1</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>151.6</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>66.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>黑龙江</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>49.1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>29.1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>14.5</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>614.0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>416.1</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>197.9</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>51.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>46.5</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>46.5</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>336.0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>39.8</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>296.2</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>21.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>江苏</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1075.2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>127.5</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>947.7</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>505.2</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>5003.3</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1283.3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>3720.0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1364.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>浙江</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>521.3</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>46.7</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>474.6</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>59.0</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>3878.0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>713.9</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>3164.1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>296.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>安徽</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>504.5</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>83.2</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>421.3</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>192.3</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>3727.6</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1369.2</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2358.5</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1143.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>福建</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>181.0</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>169.9</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>37.2</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>1055.5</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>55.2</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>1000.3</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>377.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>江西</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>313.8</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>228.8</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>85.0</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>25.3</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2306.9</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1209.9</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>1097.1</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>600.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>河南</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>310.6</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>310.6</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>49.9</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>4042.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>630.0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>3412.0</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2281.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>湖北</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>439.2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>197.8</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>241.4</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>25.6</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2926.5</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1947.0</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>979.5</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>318.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>湖南</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>266.8</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>43.1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>223.7</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>23.7</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1518.5</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>442.8</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>1075.7</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>325.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>47.6</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>16.5</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>31.2</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>204.5</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>97.8</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>106.6</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>四川</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>171.5</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>155.5</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>745.1</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>678.4</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>66.7</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>19.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>陕西</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>210.1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>14.6</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>195.5</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>96.2</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2501.5</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1834.0</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>667.5</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>347.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>甘肃</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>232.7</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>200.0</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>32.6</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>12.9</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2751.4</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2614.8</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>136.6</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>36.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>青海</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>198.0</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>195.2</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2685.0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2663.0</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>22.1</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>宁夏</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>232.1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>212.7</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>19.5</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2327.5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2183.0</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>144.5</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>新疆</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>932.6</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>931.8</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>3875.2</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>3856.5</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>18.7</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>新疆兵团</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>47.1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>273.5</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>273.5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>西藏</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>26.6</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>26.2</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>281.6</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>276.5</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>广东</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>752.7</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>348.5</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>404.3</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>44.2</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>3274.0</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>1243.6</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2030.4</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>267.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>广西</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>326.3</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>78.2</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>248.1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>1459.0</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>883.1</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>575.9</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>19.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>海南</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>159.8</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>100.3</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>59.5</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>632.3</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>414.7</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>217.5</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>23.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>贵州</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>152.0</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>122.9</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>29.1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1781.5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>1735.9</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>45.6</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>云南</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>676.3</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>608.3</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2748.1</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2546.1</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>202.0</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>29.0</t>
         </is>
       </c>
     </row>
@@ -755,7 +2259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -830,27 +2334,1275 @@
         <v>10248</v>
       </c>
       <c r="D2" t="n">
-        <v>49</v>
+        <v>4960</v>
       </c>
       <c r="E2" t="n">
-        <v>60</v>
+        <v>5288</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>1585</v>
       </c>
       <c r="G2" t="n">
-        <v>288</v>
+        <v>71293</v>
       </c>
       <c r="H2" t="n">
-        <v>1585</v>
+        <v>40342</v>
       </c>
       <c r="I2" t="n">
-        <v>71293</v>
+        <v>30951</v>
       </c>
       <c r="J2" t="n">
-        <v>40342</v>
+        <v>13184</v>
       </c>
       <c r="K2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Beijing</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G3" t="n">
+        <v>114</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>108.9</v>
+      </c>
+      <c r="J3" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="K3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>天津</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tianjin</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>119.1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="E4" t="n">
+        <v>98.3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="G4" t="n">
+        <v>608.7</v>
+      </c>
+      <c r="H4" t="n">
+        <v>319.8</v>
+      </c>
+      <c r="I4" t="n">
+        <v>288.9</v>
+      </c>
+      <c r="J4" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="K4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>河北</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hebei</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>568.2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>302.3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>265.8</v>
+      </c>
+      <c r="F5" t="n">
+        <v>98.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5984.6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>3326.2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2658.4</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1829.4</v>
+      </c>
+      <c r="K5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>山西</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Shanxi</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>352.7</v>
+      </c>
+      <c r="D6" t="n">
+        <v>209.8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>142.9</v>
+      </c>
+      <c r="F6" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2843.1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>2033.8</v>
+      </c>
+      <c r="I6" t="n">
+        <v>809.2</v>
+      </c>
+      <c r="J6" t="n">
+        <v>551.5</v>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>山东</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Shandong</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>661.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>183.4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>477.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>138.2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6353.7</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1777.2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4576.5</v>
+      </c>
+      <c r="J7" t="n">
+        <v>2699.2</v>
+      </c>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>内蒙古</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Inner Mongolia</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>466.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>394.2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2822.1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2577.2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>244.9</v>
+      </c>
+      <c r="J8" t="n">
+        <v>97.09999999999999</v>
+      </c>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>辽宁</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Liaoning</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>149.1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="E9" t="n">
+        <v>135.4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1106.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>535.1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>571.7</v>
+      </c>
+      <c r="J9" t="n">
+        <v>313.3</v>
+      </c>
+      <c r="K9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>吉林</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Jilin</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>32</v>
+      </c>
+      <c r="F10" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>511.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>360.1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>151.6</v>
+      </c>
+      <c r="J10" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="K10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>黑龙江</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Heilongjiang</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>614</v>
+      </c>
+      <c r="H11" t="n">
+        <v>416.1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>197.9</v>
+      </c>
+      <c r="J11" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="K11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Shanghai</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G12" t="n">
+        <v>336</v>
+      </c>
+      <c r="H12" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="I12" t="n">
+        <v>296.2</v>
+      </c>
+      <c r="J12" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="K12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>江苏</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Jiangsu</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1075.2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>947.7</v>
+      </c>
+      <c r="F13" t="n">
+        <v>505.2</v>
+      </c>
+      <c r="G13" t="n">
+        <v>5003.3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1283.3</v>
+      </c>
+      <c r="I13" t="n">
+        <v>3720</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1364.5</v>
+      </c>
+      <c r="K13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>浙江</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Zhejiang</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>521.3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="E14" t="n">
+        <v>474.6</v>
+      </c>
+      <c r="F14" t="n">
+        <v>59</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3878</v>
+      </c>
+      <c r="H14" t="n">
+        <v>713.9</v>
+      </c>
+      <c r="I14" t="n">
+        <v>3164.1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>296.1</v>
+      </c>
+      <c r="K14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>安徽</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Anhui</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>504.5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="E15" t="n">
+        <v>421.3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>192.3</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3727.6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1369.2</v>
+      </c>
+      <c r="I15" t="n">
+        <v>2358.5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1143.7</v>
+      </c>
+      <c r="K15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>福建</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Fujian</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>181</v>
+      </c>
+      <c r="D16" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>169.9</v>
+      </c>
+      <c r="F16" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1055.5</v>
+      </c>
+      <c r="H16" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1000.3</v>
+      </c>
+      <c r="J16" t="n">
+        <v>377.6</v>
+      </c>
+      <c r="K16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>江西</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Jiangxi</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>313.8</v>
+      </c>
+      <c r="D17" t="n">
+        <v>228.8</v>
+      </c>
+      <c r="E17" t="n">
+        <v>85</v>
+      </c>
+      <c r="F17" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2306.9</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1209.9</v>
+      </c>
+      <c r="I17" t="n">
+        <v>1097.1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>600</v>
+      </c>
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>河南</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Henan</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>310.6</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>310.6</v>
+      </c>
+      <c r="F18" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="G18" t="n">
+        <v>4042</v>
+      </c>
+      <c r="H18" t="n">
+        <v>630</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3412</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2281.2</v>
+      </c>
+      <c r="K18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>湖北</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Hubei</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>439.2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>197.8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>241.4</v>
+      </c>
+      <c r="F19" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2926.5</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1947</v>
+      </c>
+      <c r="I19" t="n">
+        <v>979.5</v>
+      </c>
+      <c r="J19" t="n">
+        <v>318</v>
+      </c>
+      <c r="K19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>湖南</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Hunan</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>266.8</v>
+      </c>
+      <c r="D20" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>223.7</v>
+      </c>
+      <c r="F20" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1518.5</v>
+      </c>
+      <c r="H20" t="n">
+        <v>442.8</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1075.7</v>
+      </c>
+      <c r="J20" t="n">
+        <v>325.4</v>
+      </c>
+      <c r="K20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Chongqing</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="D21" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G21" t="n">
+        <v>204.5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="I21" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="J21" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>四川</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Sichuan</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>171.5</v>
+      </c>
+      <c r="D22" t="n">
+        <v>155.5</v>
+      </c>
+      <c r="E22" t="n">
+        <v>16</v>
+      </c>
+      <c r="F22" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G22" t="n">
+        <v>745.1</v>
+      </c>
+      <c r="H22" t="n">
+        <v>678.4</v>
+      </c>
+      <c r="I22" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J22" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="K22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>陕西</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Shaanxi</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>210.1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="E23" t="n">
+        <v>195.5</v>
+      </c>
+      <c r="F23" t="n">
+        <v>96.2</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2501.5</v>
+      </c>
+      <c r="H23" t="n">
+        <v>1834</v>
+      </c>
+      <c r="I23" t="n">
+        <v>667.5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>347.8</v>
+      </c>
+      <c r="K23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>甘肃</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Gansu</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>232.7</v>
+      </c>
+      <c r="D24" t="n">
+        <v>200</v>
+      </c>
+      <c r="E24" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="F24" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2751.4</v>
+      </c>
+      <c r="H24" t="n">
+        <v>2614.8</v>
+      </c>
+      <c r="I24" t="n">
+        <v>136.6</v>
+      </c>
+      <c r="J24" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="K24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>青海</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Qinghai</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>198</v>
+      </c>
+      <c r="D25" t="n">
+        <v>195.2</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2685</v>
+      </c>
+      <c r="H25" t="n">
+        <v>2663</v>
+      </c>
+      <c r="I25" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>宁夏</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ningxia</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>232.1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>212.7</v>
+      </c>
+      <c r="E26" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F26" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2327.5</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2183</v>
+      </c>
+      <c r="I26" t="n">
+        <v>144.5</v>
+      </c>
+      <c r="J26" t="n">
+        <v>12</v>
+      </c>
+      <c r="K26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>新疆</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Xinjiang</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>932.6</v>
+      </c>
+      <c r="D27" t="n">
+        <v>931.8</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>3875.2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>3856.5</v>
+      </c>
+      <c r="I27" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="K27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>新疆兵团</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Xinjiang Production and Construction Corps</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>273.5</v>
+      </c>
+      <c r="H28" t="n">
+        <v>273.5</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>西藏</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Tibet</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>281.6</v>
+      </c>
+      <c r="H29" t="n">
+        <v>276.5</v>
+      </c>
+      <c r="I29" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>广东</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>752.7</v>
+      </c>
+      <c r="D30" t="n">
+        <v>348.5</v>
+      </c>
+      <c r="E30" t="n">
+        <v>404.3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="G30" t="n">
+        <v>3274</v>
+      </c>
+      <c r="H30" t="n">
+        <v>1243.6</v>
+      </c>
+      <c r="I30" t="n">
+        <v>2030.4</v>
+      </c>
+      <c r="J30" t="n">
+        <v>267.2</v>
+      </c>
+      <c r="K30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>广西</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Guangxi</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>326.3</v>
+      </c>
+      <c r="D31" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>248.1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1459</v>
+      </c>
+      <c r="H31" t="n">
+        <v>883.1</v>
+      </c>
+      <c r="I31" t="n">
+        <v>575.9</v>
+      </c>
+      <c r="J31" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="K31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>海南</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Hainan</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>159.8</v>
+      </c>
+      <c r="D32" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>632.3</v>
+      </c>
+      <c r="H32" t="n">
+        <v>414.7</v>
+      </c>
+      <c r="I32" t="n">
+        <v>217.5</v>
+      </c>
+      <c r="J32" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="K32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>贵州</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Guizhou</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>152</v>
+      </c>
+      <c r="D33" t="n">
+        <v>122.9</v>
+      </c>
+      <c r="E33" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1781.5</v>
+      </c>
+      <c r="H33" t="n">
+        <v>1735.9</v>
+      </c>
+      <c r="I33" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="J33" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>云南</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Yunnan</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>676.3</v>
+      </c>
+      <c r="D34" t="n">
+        <v>608.3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>68</v>
+      </c>
+      <c r="F34" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2748.1</v>
+      </c>
+      <c r="H34" t="n">
+        <v>2546.1</v>
+      </c>
+      <c r="I34" t="n">
+        <v>202</v>
+      </c>
+      <c r="J34" t="n">
+        <v>29</v>
+      </c>
+      <c r="K34" t="b">
         <v>0</v>
       </c>
     </row>
@@ -865,7 +3617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1054,27 +3806,1275 @@
         <v>10248</v>
       </c>
       <c r="D4" t="n">
-        <v>49</v>
+        <v>4960</v>
       </c>
       <c r="E4" t="n">
-        <v>60</v>
+        <v>5288</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>1585</v>
       </c>
       <c r="G4" t="n">
-        <v>288</v>
+        <v>71293</v>
       </c>
       <c r="H4" t="n">
-        <v>1585</v>
+        <v>40342</v>
       </c>
       <c r="I4" t="n">
-        <v>71293</v>
+        <v>30951</v>
       </c>
       <c r="J4" t="n">
-        <v>40342</v>
+        <v>13184</v>
       </c>
       <c r="K4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>北京</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Beijing</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G5" t="n">
+        <v>114</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>108.9</v>
+      </c>
+      <c r="J5" t="n">
+        <v>34.4</v>
+      </c>
+      <c r="K5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>天津</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Tianjin</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>119.1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>20.9</v>
+      </c>
+      <c r="E6" t="n">
+        <v>98.3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="G6" t="n">
+        <v>608.7</v>
+      </c>
+      <c r="H6" t="n">
+        <v>319.8</v>
+      </c>
+      <c r="I6" t="n">
+        <v>288.9</v>
+      </c>
+      <c r="J6" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>河北</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Hebei</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>568.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>302.3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>265.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>98.2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5984.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>3326.2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2658.4</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1829.4</v>
+      </c>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>山西</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Shanxi</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>352.7</v>
+      </c>
+      <c r="D8" t="n">
+        <v>209.8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>142.9</v>
+      </c>
+      <c r="F8" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2843.1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2033.8</v>
+      </c>
+      <c r="I8" t="n">
+        <v>809.2</v>
+      </c>
+      <c r="J8" t="n">
+        <v>551.5</v>
+      </c>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>山东</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Shandong</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>661.2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>183.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>477.8</v>
+      </c>
+      <c r="F9" t="n">
+        <v>138.2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>6353.7</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1777.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>4576.5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2699.2</v>
+      </c>
+      <c r="K9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>内蒙古</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Inner Mongolia</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>466.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>394.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2822.1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2577.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>244.9</v>
+      </c>
+      <c r="J10" t="n">
+        <v>97.09999999999999</v>
+      </c>
+      <c r="K10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>辽宁</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Liaoning</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>149.1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="E11" t="n">
+        <v>135.4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>95.3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1106.8</v>
+      </c>
+      <c r="H11" t="n">
+        <v>535.1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>571.7</v>
+      </c>
+      <c r="J11" t="n">
+        <v>313.3</v>
+      </c>
+      <c r="K11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>吉林</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Jilin</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>51.9</v>
+      </c>
+      <c r="D12" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="E12" t="n">
+        <v>32</v>
+      </c>
+      <c r="F12" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G12" t="n">
+        <v>511.7</v>
+      </c>
+      <c r="H12" t="n">
+        <v>360.1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>151.6</v>
+      </c>
+      <c r="J12" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="K12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>黑龙江</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Heilongjiang</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>20</v>
+      </c>
+      <c r="E13" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>614</v>
+      </c>
+      <c r="H13" t="n">
+        <v>416.1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>197.9</v>
+      </c>
+      <c r="J13" t="n">
+        <v>51.4</v>
+      </c>
+      <c r="K13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>上海</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Shanghai</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G14" t="n">
+        <v>336</v>
+      </c>
+      <c r="H14" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="I14" t="n">
+        <v>296.2</v>
+      </c>
+      <c r="J14" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="K14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>江苏</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Jiangsu</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1075.2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>947.7</v>
+      </c>
+      <c r="F15" t="n">
+        <v>505.2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>5003.3</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1283.3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3720</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1364.5</v>
+      </c>
+      <c r="K15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>浙江</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Zhejiang</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>521.3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>474.6</v>
+      </c>
+      <c r="F16" t="n">
+        <v>59</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3878</v>
+      </c>
+      <c r="H16" t="n">
+        <v>713.9</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3164.1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>296.1</v>
+      </c>
+      <c r="K16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>安徽</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Anhui</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>504.5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>83.2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>421.3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>192.3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>3727.6</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1369.2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2358.5</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1143.7</v>
+      </c>
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>福建</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Fujian</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>181</v>
+      </c>
+      <c r="D18" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>169.9</v>
+      </c>
+      <c r="F18" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1055.5</v>
+      </c>
+      <c r="H18" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1000.3</v>
+      </c>
+      <c r="J18" t="n">
+        <v>377.6</v>
+      </c>
+      <c r="K18" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>江西</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Jiangxi</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>313.8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>228.8</v>
+      </c>
+      <c r="E19" t="n">
+        <v>85</v>
+      </c>
+      <c r="F19" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="G19" t="n">
+        <v>2306.9</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1209.9</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1097.1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>600</v>
+      </c>
+      <c r="K19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>河南</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Henan</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>310.6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>310.6</v>
+      </c>
+      <c r="F20" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="G20" t="n">
+        <v>4042</v>
+      </c>
+      <c r="H20" t="n">
+        <v>630</v>
+      </c>
+      <c r="I20" t="n">
+        <v>3412</v>
+      </c>
+      <c r="J20" t="n">
+        <v>2281.2</v>
+      </c>
+      <c r="K20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>湖北</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hubei</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>439.2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>197.8</v>
+      </c>
+      <c r="E21" t="n">
+        <v>241.4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>2926.5</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1947</v>
+      </c>
+      <c r="I21" t="n">
+        <v>979.5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>318</v>
+      </c>
+      <c r="K21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>湖南</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Hunan</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>266.8</v>
+      </c>
+      <c r="D22" t="n">
+        <v>43.1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>223.7</v>
+      </c>
+      <c r="F22" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1518.5</v>
+      </c>
+      <c r="H22" t="n">
+        <v>442.8</v>
+      </c>
+      <c r="I22" t="n">
+        <v>1075.7</v>
+      </c>
+      <c r="J22" t="n">
+        <v>325.4</v>
+      </c>
+      <c r="K22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Chongqing</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="D23" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="E23" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G23" t="n">
+        <v>204.5</v>
+      </c>
+      <c r="H23" t="n">
+        <v>97.8</v>
+      </c>
+      <c r="I23" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="J23" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="K23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>四川</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Sichuan</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>171.5</v>
+      </c>
+      <c r="D24" t="n">
+        <v>155.5</v>
+      </c>
+      <c r="E24" t="n">
+        <v>16</v>
+      </c>
+      <c r="F24" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="G24" t="n">
+        <v>745.1</v>
+      </c>
+      <c r="H24" t="n">
+        <v>678.4</v>
+      </c>
+      <c r="I24" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="J24" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="K24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>陕西</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Shaanxi</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>210.1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="E25" t="n">
+        <v>195.5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>96.2</v>
+      </c>
+      <c r="G25" t="n">
+        <v>2501.5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>1834</v>
+      </c>
+      <c r="I25" t="n">
+        <v>667.5</v>
+      </c>
+      <c r="J25" t="n">
+        <v>347.8</v>
+      </c>
+      <c r="K25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>甘肃</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gansu</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>232.7</v>
+      </c>
+      <c r="D26" t="n">
+        <v>200</v>
+      </c>
+      <c r="E26" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="F26" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2751.4</v>
+      </c>
+      <c r="H26" t="n">
+        <v>2614.8</v>
+      </c>
+      <c r="I26" t="n">
+        <v>136.6</v>
+      </c>
+      <c r="J26" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="K26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>青海</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Qinghai</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>198</v>
+      </c>
+      <c r="D27" t="n">
+        <v>195.2</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2685</v>
+      </c>
+      <c r="H27" t="n">
+        <v>2663</v>
+      </c>
+      <c r="I27" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="J27" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K27" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>宁夏</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ningxia</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>232.1</v>
+      </c>
+      <c r="D28" t="n">
+        <v>212.7</v>
+      </c>
+      <c r="E28" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2327.5</v>
+      </c>
+      <c r="H28" t="n">
+        <v>2183</v>
+      </c>
+      <c r="I28" t="n">
+        <v>144.5</v>
+      </c>
+      <c r="J28" t="n">
+        <v>12</v>
+      </c>
+      <c r="K28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>新疆</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Xinjiang</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>932.6</v>
+      </c>
+      <c r="D29" t="n">
+        <v>931.8</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>3875.2</v>
+      </c>
+      <c r="H29" t="n">
+        <v>3856.5</v>
+      </c>
+      <c r="I29" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="K29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>新疆兵团</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Xinjiang Production and Construction Corps</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>273.5</v>
+      </c>
+      <c r="H30" t="n">
+        <v>273.5</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>西藏</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Tibet</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="D31" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>281.6</v>
+      </c>
+      <c r="H31" t="n">
+        <v>276.5</v>
+      </c>
+      <c r="I31" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>广东</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Guangdong</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>752.7</v>
+      </c>
+      <c r="D32" t="n">
+        <v>348.5</v>
+      </c>
+      <c r="E32" t="n">
+        <v>404.3</v>
+      </c>
+      <c r="F32" t="n">
+        <v>44.2</v>
+      </c>
+      <c r="G32" t="n">
+        <v>3274</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1243.6</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2030.4</v>
+      </c>
+      <c r="J32" t="n">
+        <v>267.2</v>
+      </c>
+      <c r="K32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>广西</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Guangxi</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>326.3</v>
+      </c>
+      <c r="D33" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="E33" t="n">
+        <v>248.1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G33" t="n">
+        <v>1459</v>
+      </c>
+      <c r="H33" t="n">
+        <v>883.1</v>
+      </c>
+      <c r="I33" t="n">
+        <v>575.9</v>
+      </c>
+      <c r="J33" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="K33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>海南</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Hainan</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>159.8</v>
+      </c>
+      <c r="D34" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="E34" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G34" t="n">
+        <v>632.3</v>
+      </c>
+      <c r="H34" t="n">
+        <v>414.7</v>
+      </c>
+      <c r="I34" t="n">
+        <v>217.5</v>
+      </c>
+      <c r="J34" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="K34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>贵州</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Guizhou</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>152</v>
+      </c>
+      <c r="D35" t="n">
+        <v>122.9</v>
+      </c>
+      <c r="E35" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1781.5</v>
+      </c>
+      <c r="H35" t="n">
+        <v>1735.9</v>
+      </c>
+      <c r="I35" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="J35" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="K35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>云南</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Yunnan</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>676.3</v>
+      </c>
+      <c r="D36" t="n">
+        <v>608.3</v>
+      </c>
+      <c r="E36" t="n">
+        <v>68</v>
+      </c>
+      <c r="F36" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2748.1</v>
+      </c>
+      <c r="H36" t="n">
+        <v>2546.1</v>
+      </c>
+      <c r="I36" t="n">
+        <v>202</v>
+      </c>
+      <c r="J36" t="n">
+        <v>29</v>
+      </c>
+      <c r="K36" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>